<commit_message>
Actualizacion datos REM VIH  0931
</commit_message>
<xml_diff>
--- a/2025/salida/P11_2025.xlsx
+++ b/2025/salida/P11_2025.xlsx
@@ -21,16 +21,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,292 +481,292 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Región</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Servicio de Salud</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Comuna</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Establecimiento</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Codigo DEIS</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Prestación</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Detalle de prestación</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Año</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Codigo Servicio REM</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Codigo Comuna REM</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>COL01 - TOTAL - Ambos sexos</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>COL02 - TOTAL - Hombres</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>COL03 - TOTAL - Mujeres</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>COL04 - RANGO ETARIO Y SEXO - Menor 1 Año - Hombres</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>COL05 - RANGO ETARIO Y SEXO - Menor 1 Año - Mujeres</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>COL06 - RANGO ETARIO Y SEXO - 1 año - Hombres</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>COL07 - RANGO ETARIO Y SEXO - 1 año - Mujeres</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>COL08 - RANGO ETARIO Y SEXO - 2 a 4 años - Hombres</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>COL09 - RANGO ETARIO Y SEXO - 2 a 4 años - Mujeres</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>COL10 - RANGO ETARIO Y SEXO - 5 a 9 años - Hombres</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>COL11 - RANGO ETARIO Y SEXO - 5 a 9 años - Mujeres</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>COL12 - RANGO ETARIO Y SEXO - 10 a 14 años - Hombres</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>COL13 - RANGO ETARIO Y SEXO - 10 a 14 años - Mujeres</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>COL14 - RANGO ETARIO Y SEXO - 15 a 19 años - Hombres</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>COL15 - RANGO ETARIO Y SEXO - 15 a 19 años - Mujeres</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>COL16 - RANGO ETARIO Y SEXO - 20 a 24 años - Hombres</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>COL17 - RANGO ETARIO Y SEXO - 20 a 24 años - Mujeres</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>COL18 - RANGO ETARIO Y SEXO - 25 a 29 años - Hombres</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>COL19 - RANGO ETARIO Y SEXO - 25 a 29 años - Mujeres</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>COL20 - RANGO ETARIO Y SEXO - 30 a 34 años - Hombres</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>COL21 - RANGO ETARIO Y SEXO - 30 a 34 años - Mujeres</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>COL22 - RANGO ETARIO Y SEXO - 35 a 39 años - Hombres</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>COL23 - RANGO ETARIO Y SEXO - 35 a 39 años - Mujeres</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>COL24 - RANGO ETARIO Y SEXO - 40 a 44 años - Hombres</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>COL25 - RANGO ETARIO Y SEXO - 40 a 44 años - Mujeres</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>COL26 - RANGO ETARIO Y SEXO - 45 a 49 años - Hombres</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>COL27 - RANGO ETARIO Y SEXO - 45 a 49 años - Mujeres</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>COL28 - RANGO ETARIO Y SEXO - 50 a 54 años - Hombres</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>COL29 - RANGO ETARIO Y SEXO - 50 a 54 años - Mujeres</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>COL30 - RANGO ETARIO Y SEXO - 55 a 59 años - Hombres</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>COL31 - RANGO ETARIO Y SEXO - 55 a 59 años - Mujeres</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>COL32 - RANGO ETARIO Y SEXO - 60 a 64 años - Hombres</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>COL33 - RANGO ETARIO Y SEXO - 60 a 64 años - Mujeres</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>COL34 - RANGO ETARIO Y SEXO - 65 a 69 años - Hombres</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>COL35 - RANGO ETARIO Y SEXO - 65 a 69 años - Mujeres</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>COL36 - RANGO ETARIO Y SEXO - 70 a 74 años - Hombres</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>COL37 - RANGO ETARIO Y SEXO - 70 a 74 años - Mujeres</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>COL38 - RANGO ETARIO Y SEXO - 75 a 79 años - Hombres</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>COL39 - RANGO ETARIO Y SEXO - 75 a 79 años - Mujeres</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>COL40 - RANGO ETARIO Y SEXO - 80 y más años - Hombres</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>COL41 - RANGO ETARIO Y SEXO - 80 y más años - Mujeres</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>COL42 - TRANS - Masculino</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>COL43 - TRANS - Femenino</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>COL44 - Pueblos Originarios</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>COL45 - Migrantes</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>COL46 - Niños, Niñas, Adolescentes y Jóvenes SENAME</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>COL47 - Niños, Niñas, Adolescentes y Jóvenes Mejor Niñez</t>
         </is>
@@ -7075,29 +7063,31 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="M42" t="n">
         <v>7</v>
       </c>
       <c r="N42" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="n">
         <v>1</v>
       </c>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
+      <c r="R42" t="n">
+        <v>1</v>
+      </c>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U42" t="n">
         <v>3</v>
       </c>
       <c r="V42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W42" t="n">
         <v>2</v>
@@ -7213,29 +7203,29 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M43" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" t="n">
-        <v>1</v>
-      </c>
+      <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
+      <c r="R43" t="n">
+        <v>1</v>
+      </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W43" t="n">
         <v>2</v>
@@ -7244,7 +7234,7 @@
         <v>2</v>
       </c>
       <c r="Y43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z43" t="n">
         <v>1</v>
@@ -10774,232 +10764,232 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Región</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Servicio de Salud</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Comuna</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Establecimiento</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Codigo DEIS</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Prestación</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Detalle de prestación</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Año</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Codigo Servicio REM</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Codigo Comuna REM</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>COL01 - TOTAL - Ambos sexos</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>COL02 - TOTAL - Hombres</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>COL03 - TOTAL - Mujeres</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>COL04 - RANGO ETARIO Y SEXO - 15 a 19 años - Hombres</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>COL05 - RANGO ETARIO Y SEXO - 15 a 19 años - Mujeres</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>COL06 - RANGO ETARIO Y SEXO - 20 a 24 años - Hombres</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>COL07 - RANGO ETARIO Y SEXO - 20 a 24 años - Mujeres</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>COL08 - RANGO ETARIO Y SEXO - 25 a 29 años - Hombres</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>COL09 - RANGO ETARIO Y SEXO - 25 a 29 años - Mujeres</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>COL10 - RANGO ETARIO Y SEXO - 30 a 34 años - Hombres</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>COL11 - RANGO ETARIO Y SEXO - 30 a 34 años - Mujeres</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>COL12 - RANGO ETARIO Y SEXO - 35 a 39 años - Hombres</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>COL13 - RANGO ETARIO Y SEXO - 35 a 39 años - Mujeres</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>COL14 - RANGO ETARIO Y SEXO - 40 a 44 años - Hombres</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>COL15 - RANGO ETARIO Y SEXO - 40 a 44 años - Mujeres</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>COL16 - RANGO ETARIO Y SEXO - 45 a 49 años - Hombres</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>COL17 - RANGO ETARIO Y SEXO - 45 a 49 años - Mujeres</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>COL18 - RANGO ETARIO Y SEXO - 50 a 54 años - Hombres</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>COL19 - RANGO ETARIO Y SEXO - 50 a 54 años - Mujeres</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>COL20 - RANGO ETARIO Y SEXO - 55 a 59 años - Hombres</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>COL21 - RANGO ETARIO Y SEXO - 55 a 59 años - Mujeres</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>COL22 - RANGO ETARIO Y SEXO - 60 a 64 años - Hombres</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>COL23 - RANGO ETARIO Y SEXO - 60 a 64 años - Mujeres</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>COL24 - RANGO ETARIO Y SEXO - 65 a 69 años - Hombres</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>COL25 - RANGO ETARIO Y SEXO - 65 a 69 años - Mujeres</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>COL26 - RANGO ETARIO Y SEXO - 70 a 74 años - Hombres</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>COL27 - RANGO ETARIO Y SEXO - 70 a 74 años - Mujeres</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>COL28 - RANGO ETARIO Y SEXO - 75 a 79 años - Hombres</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>COL29 - RANGO ETARIO Y SEXO - 75 a 79 años - Mujeres</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>COL30 - RANGO ETARIO Y SEXO - 80 y más años - Hombres</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>COL31 - RANGO ETARIO Y SEXO - 80 y más años - Mujeres</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>COL32 - TRANS - Masculino</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>COL33 - TRANS - Femenino</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>COL34 - Pueblos Originarios</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>COL35 - Migrantes</t>
         </is>

</xml_diff>